<commit_message>
배포판 자동 동기화 — 49e3968 (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -57,11 +57,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,9 +461,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -465,9 +469,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -475,9 +477,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -485,9 +485,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -495,9 +493,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -505,9 +501,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -515,9 +509,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -525,9 +517,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -535,9 +525,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -580,9 +568,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -653,9 +639,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -681,14 +665,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK46"/>
+  <dimension ref="A1:AL46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
@@ -721,109 +705,114 @@
           <t>가능근무</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>야간리더</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>전입</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>전입일</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="I2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="J2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="K2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="L2" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="L2" s="1" t="n">
+      <c r="M2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="M2" s="1" t="n">
+      <c r="N2" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="O2" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="O2" s="1" t="n">
+      <c r="P2" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="P2" s="1" t="n">
+      <c r="Q2" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="Q2" s="1" t="n">
+      <c r="R2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="R2" s="1" t="n">
+      <c r="S2" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="S2" s="1" t="n">
+      <c r="T2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="T2" s="1" t="n">
+      <c r="U2" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="U2" s="1" t="n">
+      <c r="V2" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="V2" s="1" t="n">
+      <c r="W2" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="W2" s="1" t="n">
+      <c r="X2" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="X2" s="1" t="n">
+      <c r="Y2" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="Y2" s="1" t="n">
+      <c r="Z2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="Z2" s="1" t="n">
+      <c r="AA2" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="AA2" s="1" t="n">
+      <c r="AB2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AB2" s="1" t="n">
+      <c r="AC2" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="AC2" s="1" t="n">
+      <c r="AD2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="AD2" s="1" t="n">
+      <c r="AE2" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="AE2" s="1" t="n">
+      <c r="AF2" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="AF2" s="1" t="n">
+      <c r="AG2" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="AG2" s="1" t="n">
+      <c r="AH2" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="AH2" s="1" t="n">
+      <c r="AI2" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="AI2" s="1" t="n">
+      <c r="AJ2" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="AJ2" s="1" t="n">
+      <c r="AK2" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="AK2" s="1" t="n">
+      <c r="AL2" s="1" t="n">
         <v>30</v>
       </c>
     </row>
@@ -855,7 +844,7 @@
           <t>8A</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -878,7 +867,7 @@
           <t>D,E,N,지정</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -901,7 +890,7 @@
           <t>D,E,N,지정</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -924,7 +913,7 @@
           <t>D,E,N,prn,3N</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -947,7 +936,7 @@
           <t>prn</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -970,12 +959,12 @@
           <t>D,E</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>임부(야간 금지)</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -998,7 +987,7 @@
           <t>D,E,N,2N</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1021,7 +1010,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1044,7 +1033,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1067,7 +1056,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1090,12 +1079,12 @@
           <t>NK</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>야간전담</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1118,7 +1107,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1141,12 +1130,12 @@
           <t>NK</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>야간전담</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1169,12 +1158,12 @@
           <t>D,E</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>임부(야간 금지)</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1197,7 +1186,7 @@
           <t>D,E</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1220,7 +1209,12 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1243,7 +1237,7 @@
           <t>D,E,N,prn,지정</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1266,7 +1260,12 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1289,7 +1288,12 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1312,7 +1316,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1335,7 +1339,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1358,7 +1362,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1381,7 +1385,7 @@
           <t>D,E,N,지정</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1404,7 +1408,7 @@
           <t>D,E,N,prn</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1427,7 +1431,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1450,7 +1454,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1473,7 +1477,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1496,7 +1500,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1519,7 +1523,7 @@
           <t>D,E,N,지정</t>
         </is>
       </c>
-      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1542,7 +1546,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1565,7 +1569,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1588,7 +1592,7 @@
           <t>D,E,N,prn</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1611,7 +1615,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1634,7 +1638,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1657,7 +1661,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1680,7 +1684,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1703,7 +1707,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1726,7 +1730,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1749,7 +1753,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1772,7 +1776,7 @@
           <t>D,E,N</t>
         </is>
       </c>
-      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -1797,10 +1801,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="F4:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="전입 여부" prompt="이번 달에 새로 온 사람이면 '전입'을 고르세요. 월중 전입이면 옆 칸에 입사일을 적어주세요(비우면 1일자 전입으로 봅니다)." type="list">
+    <dataValidation sqref="G4:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="전입 여부" prompt="이번 달에 새로 온 사람이면 '전입'을 고르세요. 월중 전입이면 옆 칸에 입사일을 적어주세요(비우면 1일자 전입으로 봅니다)." type="list">
       <formula1>"전입"</formula1>
     </dataValidation>
-    <dataValidation sqref="G4:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="전입일" prompt="월중 입사면 날짜를 적어주세요 — 9월 15일에 오면 '15' · '9월 15일' · '2026-09-15' 다 됩니다. 비우면 1일자 전입입니다."/>
+    <dataValidation sqref="H4:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="전입일" prompt="월중 입사면 날짜를 적어주세요. 비우면 1일자 전입입니다."/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
배포판 자동 동기화 — 37a7047 (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -461,7 +461,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -469,7 +468,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -477,7 +475,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -485,7 +482,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -493,7 +489,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -501,7 +496,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -509,7 +503,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -517,7 +510,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -525,7 +517,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -568,7 +559,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -639,7 +629,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -1339,6 +1328,11 @@
           <t>D,E,N</t>
         </is>
       </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
@@ -1383,6 +1377,11 @@
       <c r="D26" t="inlineStr">
         <is>
           <t>D,E,N,지정</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="H26" s="2" t="n"/>

</xml_diff>

<commit_message>
배포판 자동 동기화 — 03701bf (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -461,6 +461,9 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -468,6 +471,9 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -475,169 +481,206 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>⚠ '가능근무' 칸에는 근무코드(D·E·N·prn 등) 외에 세 가지를 더 적을 수 있습니다. 2N·3N은 야간을 며칠씩 묶어 서고 싶은지입니다(안 적으면 2N). 3N은 3일씩 묶어 서므로 그 사람의 월 야간이 상한(기본 6회)으로 고정됩니다 — 3일 블록으로는 하한 4를 만들 수 없기 때문입니다. '지정'은 근무인력 표의 '지정' 인원으로 셀 수 있는 사람이라는 표시로, 그날 D·E·N·prn 중 무엇이든 서면 자동으로 한 명으로 세집니다. 셋 다 근무가 아니라 표시라서, D·E·N 같은 근무를 함께 적어야 배정됩니다.</t>
-        </is>
-      </c>
+          <t>⚠ '가능근무' 칸에는 근무코드(D·E·N·prn 등) 외에 세 가지를 더 적을 수 있습니다. 2N·3N은 야간을 며칠씩 묶어 서고 싶은지입니다(안 적으면 2N). 3N은 3일씩 묶어 서므로 그 사람의 월 야간이 상한(기본 6회)으로 고정됩니다 — 3일 블록으로는 하한 4를 만들 수 없기 때문입니다. '지정'은 근무인력 표의 '지정' 인원으로 셀 수 있는 사람이라는 표시로, 그날 D·E·N·prn 중 무엇이든 서면 자동으로 한 명으로 세집니다. 셋 다 근무코드가 아니라 표시입니다 — '지정'은 어떤 근무를 설 수 있는지 알 수 없으므로 D·E·N 같은 근무를 반드시 함께 적어야 하고(지정만 적으면 반려합니다), 2N·3N은 '야간을 이렇게 묶는다'는 뜻이라 N을 따로 안 적어도 야간 가능자로 봅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>⚠ prn 인원은 8A·9A·10A와 8H·9H·10H, 그리고 그 변형(8A*·8A◎ 등)을 한 덩어리로 셉니다 — 시작 시각만 다른 같은 근무라서입니다. 반일 근무(8AH·9AH·9H*)만 0.5명으로 세기 때문에 출력 근무표의 'prn 인원' 줄에 2.5 같은 값이 뜰 수 있습니다(반나절 선 사람을 온종일 선 것으로 세면 못 채운 날이 채운 날처럼 보이기 때문입니다).</t>
-        </is>
-      </c>
+          <t>⚠ '야간리더' 칸은 **밤을 맡길 수 있는 사람에게만 O**를 적습니다(비우면 아님). 야간에는 숙련도 4 이상이 한 명은 반드시 있어야 하는데(필수 규칙), 리더가 주간 전담인 병동에서는 밤에 세울 사람이 한두 명뿐이라 매일 밤을 채울 수가 없습니다. 이 칸에 표시된 사람은 숙련도와 상관없이 그 조건을 채운 것으로 봅니다. 쓰지 않는 병동은 전부 비워두면 지금까지와 똑같이 숙련도로만 판정합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>⚠ '전입'·'전입일' 칸 — 이번 달에 새로 온 사람은 '전입'을 고르고, 월중 입사면 입사일을 적어주세요(비우면 1일자 전입). 입사 전 날짜는 배정에서 빠집니다.</t>
-        </is>
-      </c>
+          <t>⚠ prn 인원은 8A·9A·10A와 8H·9H·10H, 그리고 그 변형(8A*·8A◎ 등)을 한 덩어리로 셉니다 — 시작 시각만 다른 같은 근무라서입니다. 반일 근무(8AH·9AH·9H*)만 0.5명으로 세기 때문에 출력 근무표의 'prn 인원' 줄에 2.5 같은 값이 뜰 수 있습니다(반나절 선 사람을 온종일 선 것으로 세면 못 채운 날이 채운 날처럼 보이기 때문입니다).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>⚠ 날짜 칸은 OCS 화면에서 그대로 복사해 붙여넣어도 됩니다 — 말일 칸 오른쪽에 딸려온 D/E/N·®·ⓡ·금월·T연·R연·부서 같은 칸은 읽지 않으니 그냥 두셔도 되고 지우셔도 됩니다.</t>
-        </is>
-      </c>
+          <t>⚠ '전입'·'전입일' 칸 — 이번 달에 새로 온 사람은 '전입'을 고르고, 월중 입사면 입사일을 적어주세요(비우면 1일자 전입). 입사 전 날짜는 배정에서 빠집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>⚠ 인원 명단 아래 이름 칸에 'B' 한 글자만 있는 구분 행과 그 아래 이름들은 B팀(신입)입니다 — 근무 배정에는 전혀 관여하지 않고 출력 근무표에 이름만 표시됩니다. 필요 없으면 그 행들을 지우고 올리세요.</t>
-        </is>
-      </c>
+          <t>⚠ 날짜 칸은 OCS 화면에서 그대로 복사해 붙여넣어도 됩니다 — 말일 칸 오른쪽에 딸려온 D/E/N·®·ⓡ·금월·T연·R연·부서 같은 칸은 읽지 않으니 그냥 두셔도 되고 지우셔도 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>⚠ 중요 — '원티드표' 시트의 A1 셀에 적힌 'YYYY년 M월'을 보고 코드가 이 파일이 몇 년 몇 월 신청분인지 자동으로 인식합니다. A1의 월 이름을 실제 신청 대상 월과 다르게 고치면(예: 파일을 복사해서 재사용하다가 안 고침) 엉뚱한 달로 인식되니, 월을 바꿀 때는 A1도 꼭 같이 맞춰주세요 — 파일명이 아니라 A1 셀 내용을 봅니다.</t>
-        </is>
-      </c>
+          <t>⚠ 인원 명단 아래 이름 칸에 'B' 한 글자만 있는 구분 행과 그 아래 이름들은 B팀(신입)입니다 — 근무 배정에는 전혀 관여하지 않고 출력 근무표에 이름만 표시됩니다. 필요 없으면 그 행들을 지우고 올리세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>표기 코드 (뒤에 별표 * 가 있어도 없어도 인식됩니다)</t>
+          <t>⚠ 중요 — '원티드표' 시트의 A1 셀에 적힌 'YYYY년 M월'을 보고 코드가 이 파일이 몇 년 몇 월 신청분인지 자동으로 인식합니다. A1의 월 이름을 실제 신청 대상 월과 다르게 고치면(예: 파일을 복사해서 재사용하다가 안 고침) 엉뚱한 달로 인식되니, 월을 바꿀 때는 A1도 꼭 같이 맞춰주세요 — 파일명이 아니라 A1 셀 내용을 봅니다.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>· 근무 희망: D / E / N / 8A / 9A / NK / prn / T(교육) / TW(반근무+반교육)</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>· 휴가유형별 희망: 연·연차(연차) / 연1·연2·연3(시간제 연차) / 연4(반차) / 조(조사) / 경(경조사) / 공(공가) / 병(병가) / 휴(휴직) / 승(승급교육) / 군(군공가)</t>
+          <t>표기 코드 (뒤에 별표 * 가 있어도 없어도 인식됩니다)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>· 단순 OFF 희망: X</t>
+          <t>· 근무 희망: D / E / N / 8A / 9A / NK / prn / T(교육) / TW(반근무+반교육)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>· 그 외 인식 못 하는 표시(포상휴가 등 특수 코드)는 업로드 후 '인식 못 한 표시' 목록으로 알려드립니다.</t>
+          <t>· 휴가유형별 희망: 연·연차(연차) / 연1·연2·연3(시간제 연차) / 연4(반차) / 조(조사) / 경(경조사) / 공(공가) / 병(병가) / 휴(휴직) / 승(승급교육) / 군(군공가)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>· 빈 칸은 신청 없음으로 건너뜁니다.</t>
+          <t>· 단순 OFF 희망: X</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>· 그 외 인식 못 하는 표시(포상휴가 등 특수 코드)는 업로드 후 '인식 못 한 표시' 목록으로 알려드립니다.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>각 코드가 배정에서 어떻게 처리되는지</t>
+          <t>· 빈 칸은 신청 없음으로 건너뜁니다.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>· 병(병가): 연속근무일수 계산에서 제외됩니다(연속근무 5일 제한에 안 걸림)</t>
-        </is>
-      </c>
+      <c r="A27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>· 휴(휴직): **적은 날짜 하루만** 제외됩니다. 월 나머지가 자동으로 채워지지 않으니 휴직·장기휴가는 쉬는 날마다 한 칸씩 적어주세요(며칠짜리인지는 파트장이 지정).</t>
+          <t>각 코드가 배정에서 어떻게 처리되는지</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  같은 방식으로 사(사사휴직)/상(상병휴직)/산전/육법/육연/R/출산도 날짜마다 적습니다.</t>
+          <t>· 병(병가): 연속근무일수 계산에서 제외됩니다(연속근무 5일 제한에 안 걸림)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>· 공/승(공가/승급교육): 휴무(OFF)와 동일하게 취급되지만 연차는 차감되지 않습니다</t>
+          <t>· 휴(휴직): **적은 날짜 하루만** 제외됩니다. 월 나머지가 자동으로 채워지지 않으니 휴직·장기휴가는 쉬는 날마다 한 칸씩 적어주세요(며칠짜리인지는 파트장이 지정).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>· 연1/연2/연3/연4(시간제/반차 연차): 몇 시간이든 하루치 연차 희망으로 집계됩니다</t>
+          <t xml:space="preserve">  같은 방식으로 사(사사휴직)/상(상병휴직)/산전/육법/육연/R/출산도 날짜마다 적습니다.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>· 군(군공가): 휴무(OFF)와 동일하게 취급되지만 잔휴에는 반영되지 않습니다</t>
+          <t>· 공/승(공가/승급교육): 휴무(OFF)와 동일하게 취급되지만 연차는 차감되지 않습니다</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>· S/(수면오프)는 이 표에 신청할 수 없습니다 — 월 야간이 6회 이상이면 프로그램이 자동으로 하루 넣어줍니다. 오프를 대신 쓰는 것이 아니라 오프와 별도로 하루가 더 생깁니다(그 달 안에서 날짜는 자유롭게 옮겨 쓰세요). 야간이 몇 회든 1개이고, 원티드로는 신청할 수 없습니다</t>
+          <t>· 연1/연2/연3/연4(시간제/반차 연차): 몇 시간이든 하루치 연차 희망으로 집계됩니다</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>· TW(반근무+반교육): 근무일수엔 포함되지만 최소인력 계산에는 제외됩니다(교육 T와 동일)</t>
+          <t>· 군(군공가): 휴무(OFF)와 동일하게 취급되지만 잔휴에는 반영되지 않습니다</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>· 9A(09시 시작): 8A와 동격으로 취급됩니다(시작 시각만 다름). 8A·9A·10A와 8H·9H·10H, 그리고 그 변형(8A*·8AH 등)은 하단 'prn 인원'에 함께 잡힙니다 — 반일 근무(8AH·9AH·9H*)만 0.5명으로 셉니다</t>
+          <t>· S/(수면오프)는 이 표에 신청할 수 없습니다 — 월 야간이 6회 이상이면 프로그램이 자동으로 하루 넣어줍니다. 오프를 대신 쓰는 것이 아니라 오프와 별도로 하루가 더 생깁니다(그 달 안에서 날짜는 자유롭게 옮겨 쓰세요). 야간이 몇 회든 1개이고, 원티드로는 신청할 수 없습니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>· TW(반근무+반교육): 근무일수엔 포함되지만 최소인력 계산에는 제외됩니다(교육 T와 동일)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>· 9A(09시 시작): 8A와 동격으로 취급됩니다(시작 시각만 다름). 8A·9A·10A와 8H·9H·10H, 그리고 그 변형(8A*·8AH 등)은 하단 'prn 인원'에 함께 잡힙니다 — 반일 근무(8AH·9AH·9H*)만 0.5명으로 셉니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>가장 쉬운 사용법</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>이번 달 근무표를 아무 값이나 넣어 한 번 생성해서 빈 그리드 모양(입력②와 같은 모양)을 받은 뒤, 그 위에 표시만 채워서 다시 올려도 됩니다.</t>
         </is>

</xml_diff>